<commit_message>
fix: clarify occupancy metric is guest-nights, not calendar days
</commit_message>
<xml_diff>
--- a/proyectos/la-nuite/Proyecciones La Nuit 2026.xlsx
+++ b/proyectos/la-nuite/Proyecciones La Nuit 2026.xlsx
@@ -1,19 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be54658ce2bde5a7/Desktop/FELO/pruebavscode/pruebavscode/proyectos/la-nuite/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_AAF1A10A40C9F263B21A8F82AA70FE541B14183E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31BC6199-C6C1-4704-A87B-D9514B3C8CC0}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen de exportación" sheetId="1" r:id="rId5"/>
-    <sheet name="Proy. X Etapas - Proyecciones f" sheetId="2" r:id="rId6"/>
-    <sheet name="Rentabilidad" sheetId="3" r:id="rId7"/>
+    <sheet name="Resumen de exportación" sheetId="1" r:id="rId1"/>
+    <sheet name="Proy. X Etapas - Proyecciones f" sheetId="2" r:id="rId2"/>
+    <sheet name="Rentabilidad" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -35,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <si>
     <t>Este documento se exportó de Numbers. Cada tabla se convirtió en una hoja de cálculo de Excel. Los demás objetos de las hojas de Numbers se colocaron en distintas hojas de cálculo. Recuerda que el cálculo de fórmulas puede ser diferente en Excel.</t>
   </si>
@@ -66,7 +88,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -75,7 +97,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -86,7 +108,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -95,7 +117,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -106,7 +128,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -115,7 +137,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -126,7 +148,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -135,7 +157,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -146,7 +168,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -155,7 +177,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -169,7 +191,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -178,7 +200,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -189,7 +211,7 @@
   <si>
     <r>
       <rPr>
-        <b val="1"/>
+        <b/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -198,7 +220,7 @@
     </r>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="10"/>
         <color indexed="15"/>
         <rFont val="Helvetica Neue"/>
@@ -276,16 +298,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
-    <numFmt numFmtId="0" formatCode="General"/>
-    <numFmt numFmtId="59" formatCode="&quot;$&quot; #,##0"/>
-    <numFmt numFmtId="60" formatCode="[$$-409] #,##0"/>
-    <numFmt numFmtId="61" formatCode="#,##0.0000%"/>
-    <numFmt numFmtId="62" formatCode="#,##0%"/>
-    <numFmt numFmtId="63" formatCode="#,##0.00%"/>
-    <numFmt numFmtId="64" formatCode="&quot;$&quot; #,##0.00"/>
-    <numFmt numFmtId="65" formatCode="0.0000%"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="7">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="165" formatCode="[$$-409]\ #,##0"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0000%"/>
+    <numFmt numFmtId="167" formatCode="#,##0%"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00%"/>
+    <numFmt numFmtId="169" formatCode="&quot;$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="170" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -304,73 +325,73 @@
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="12"/>
       <color indexed="11"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="10"/>
       <color indexed="15"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="10"/>
       <color indexed="15"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="10"/>
       <color indexed="17"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Garamond"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="12"/>
       <color indexed="19"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="12"/>
       <color indexed="21"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="12"/>
       <color indexed="22"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="9"/>
       <color indexed="15"/>
       <name val="Helvetica Neue"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="12"/>
       <color indexed="17"/>
       <name val="Garamond"/>
@@ -467,11 +488,38 @@
       <right style="thin">
         <color indexed="13"/>
       </right>
-      <top>
-        <color indexed="8"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="13"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="13"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
       </top>
-      <bottom>
-        <color indexed="8"/>
+      <bottom style="thin">
+        <color indexed="13"/>
       </bottom>
       <diagonal/>
     </border>
@@ -479,29 +527,36 @@
       <left style="thin">
         <color indexed="13"/>
       </left>
-      <right>
-        <color indexed="8"/>
+      <right style="thin">
+        <color indexed="14"/>
       </right>
-      <top>
-        <color indexed="8"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="14"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
       </top>
-      <bottom>
-        <color indexed="8"/>
+      <bottom style="thin">
+        <color indexed="13"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left>
-        <color indexed="8"/>
-      </left>
-      <right>
-        <color indexed="8"/>
-      </right>
-      <top>
-        <color indexed="8"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="13"/>
       </top>
-      <bottom>
-        <color indexed="8"/>
+      <bottom style="thin">
+        <color indexed="13"/>
       </bottom>
       <diagonal/>
     </border>
@@ -513,25 +568,10 @@
         <color indexed="13"/>
       </right>
       <top style="thin">
-        <color indexed="14"/>
+        <color indexed="13"/>
       </top>
       <bottom style="thin">
         <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="14"/>
-      </right>
-      <top>
-        <color indexed="8"/>
-      </top>
-      <bottom>
-        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
@@ -543,7 +583,7 @@
         <color indexed="13"/>
       </right>
       <top style="thin">
-        <color indexed="14"/>
+        <color indexed="13"/>
       </top>
       <bottom style="thin">
         <color indexed="13"/>
@@ -551,105 +591,38 @@
       <diagonal/>
     </border>
     <border>
-      <left>
-        <color indexed="8"/>
-      </left>
-      <right>
-        <color indexed="8"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="13"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="13"/>
       </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="13"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="13"/>
       </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="14"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left>
-        <color indexed="8"/>
-      </left>
-      <right>
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom>
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left>
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top>
-        <color indexed="8"/>
-      </top>
-      <bottom>
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left>
-        <color indexed="8"/>
-      </left>
-      <right>
-        <color indexed="8"/>
-      </right>
-      <top>
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left>
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top>
-        <color indexed="8"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color indexed="14"/>
       </bottom>
@@ -687,247 +660,247 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="79">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="0" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="61" fontId="7" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="62" fontId="4" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="0" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="63" fontId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="62" fontId="4" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="10" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="62" fontId="10" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="62" fontId="4" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="5" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="11" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="62" fontId="11" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="8" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="12" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="62" fontId="12" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="9" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="64" fontId="15" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="15" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="15" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="65" fontId="15" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="5" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="64" fontId="15" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="60" fontId="15" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="15" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="15" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -937,37 +910,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ff5e88b1"/>
-      <rgbColor rgb="ffeef3f4"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffbdc0bf"/>
-      <rgbColor rgb="ffa5a5a5"/>
-      <rgbColor rgb="ff3f3f3f"/>
-      <rgbColor rgb="fffefffe"/>
-      <rgbColor rgb="ffdbdbdb"/>
-      <rgbColor rgb="ff5e5e5e"/>
-      <rgbColor rgb="ffff968c"/>
-      <rgbColor rgb="fffe634d"/>
-      <rgbColor rgb="ff1cb000"/>
-      <rgbColor rgb="ff017000"/>
-      <rgbColor rgb="ff960d52"/>
-      <rgbColor rgb="ff919191"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FF5E88B1"/>
+      <rgbColor rgb="FFEEF3F4"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFBDC0BF"/>
+      <rgbColor rgb="FFA5A5A5"/>
+      <rgbColor rgb="FF3F3F3F"/>
+      <rgbColor rgb="FFFEFFFE"/>
+      <rgbColor rgb="FFDBDBDB"/>
+      <rgbColor rgb="FF5E5E5E"/>
+      <rgbColor rgb="FFFF968C"/>
+      <rgbColor rgb="FFFE634D"/>
+      <rgbColor rgb="FF1CB000"/>
+      <rgbColor rgb="FF017000"/>
+      <rgbColor rgb="FF960D52"/>
+      <rgbColor rgb="FF919191"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Blank">
   <a:themeElements>
     <a:clrScheme name="Blank">
       <a:dk1>
@@ -1166,7 +1187,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1184,7 +1205,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1200" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1213,7 +1234,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1238,7 +1259,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1263,7 +1284,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1288,7 +1309,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1313,7 +1334,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1338,7 +1359,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1363,7 +1384,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1388,7 +1409,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1413,7 +1434,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1426,9 +1447,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -1445,7 +1472,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1463,7 +1490,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1488,7 +1515,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1513,7 +1540,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1538,7 +1565,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1563,7 +1590,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1588,7 +1615,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1613,7 +1640,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1638,7 +1665,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1663,7 +1690,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1688,7 +1715,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1701,9 +1728,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1717,7 +1750,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="50800" tIns="50800" rIns="50800" bIns="50800" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1735,7 +1768,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1764,7 +1797,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1789,7 +1822,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1814,7 +1847,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1839,7 +1872,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1864,7 +1897,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1889,7 +1922,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1914,7 +1947,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1939,7 +1972,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1964,7 +1997,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1977,71 +2010,79 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B3:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="13.05" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="4" width="33.6016" customWidth="1"/>
+    <col min="2" max="4" width="33.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" ht="50" customHeight="1">
-      <c r="B3" t="s" s="1">
+    <row r="3" spans="2:4" ht="49.95" customHeight="1">
+      <c r="B3" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="C3"/>
-      <c r="D3"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
     </row>
-    <row r="7">
-      <c r="B7" t="s" s="2">
+    <row r="7" spans="2:4" ht="34.799999999999997">
+      <c r="B7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C7" t="s" s="2">
+      <c r="C7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D7" t="s" s="2">
+      <c r="D7" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" t="s" s="3">
+    <row r="9" spans="2:4" ht="15">
+      <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
-    <row r="10">
-      <c r="B10" s="4"/>
-      <c r="C10" t="s" s="4">
+    <row r="10" spans="2:4" ht="30">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D10" t="s" s="5">
+      <c r="D10" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" t="s" s="3">
+    <row r="11" spans="2:4" ht="15">
+      <c r="B11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
     </row>
-    <row r="12">
-      <c r="B12" s="4"/>
-      <c r="C12" t="s" s="4">
+    <row r="12" spans="2:4" ht="15">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D12" t="s" s="5">
+      <c r="D12" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2050,495 +2091,497 @@
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D10" location="'Proy. X Etapas - Proyecciones f'!R2C1" tooltip="" display="Proy. X Etapas - Proyecciones f"/>
-    <hyperlink ref="D12" location="'Rentabilidad'!R2C1" tooltip="" display="Rentabilidad"/>
+    <hyperlink ref="D10" location="'Proy. X Etapas - Proyecciones f'!R2C1" display="Proy. X Etapas - Proyecciones f" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D12" location="'Rentabilidad'!R2C1" display="Rentabilidad" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:Q15"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Q15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="19.875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="2.24219" style="6" customWidth="1"/>
-    <col min="3" max="3" width="9.33594" style="6" customWidth="1"/>
-    <col min="4" max="5" width="16.3516" style="6" customWidth="1"/>
-    <col min="6" max="6" width="2.53906" style="6" customWidth="1"/>
-    <col min="7" max="12" width="16.3516" style="6" customWidth="1"/>
-    <col min="13" max="13" width="13.2969" style="6" customWidth="1"/>
-    <col min="14" max="14" width="2.85938" style="6" customWidth="1"/>
-    <col min="15" max="15" width="13.2969" style="6" customWidth="1"/>
-    <col min="16" max="16" width="1.66406" style="6" customWidth="1"/>
-    <col min="17" max="17" width="13.2969" style="6" customWidth="1"/>
-    <col min="18" max="16384" width="16.3516" style="6" customWidth="1"/>
+    <col min="1" max="1" width="19.88671875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="2.21875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="16.33203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="2.5546875" style="5" customWidth="1"/>
+    <col min="7" max="12" width="16.33203125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" style="5" customWidth="1"/>
+    <col min="14" max="14" width="2.88671875" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.33203125" style="5" customWidth="1"/>
+    <col min="16" max="16" width="1.6640625" style="5" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="5" customWidth="1"/>
+    <col min="18" max="18" width="16.33203125" style="5" customWidth="1"/>
+    <col min="19" max="16384" width="16.33203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.65" customHeight="1">
-      <c r="A1" t="s" s="7">
+    <row r="1" spans="1:17" ht="27.6" customHeight="1">
+      <c r="A1" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
     </row>
-    <row r="2" ht="32.25" customHeight="1">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" t="s" s="10">
+    <row r="2" spans="1:17" ht="32.25" customHeight="1">
+      <c r="A2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s" s="10">
+      <c r="D2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s" s="10">
+      <c r="E2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="11"/>
-      <c r="G2" t="s" s="10">
+      <c r="F2" s="9"/>
+      <c r="G2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H2" t="s" s="10">
+      <c r="H2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s" s="10">
+      <c r="I2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s" s="10">
+      <c r="J2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="K2" t="s" s="10">
+      <c r="K2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="L2" t="s" s="10">
+      <c r="L2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="M2" t="s" s="10">
+      <c r="M2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="9"/>
-      <c r="O2" t="s" s="12">
+      <c r="N2" s="7"/>
+      <c r="O2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="14"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="12"/>
     </row>
-    <row r="3" ht="32.55" customHeight="1">
-      <c r="A3" t="s" s="15">
+    <row r="3" spans="1:17" ht="32.549999999999997" customHeight="1">
+      <c r="A3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="17">
+      <c r="B3" s="14"/>
+      <c r="C3" s="15">
         <v>4</v>
       </c>
-      <c r="D3" s="18">
+      <c r="D3" s="16">
         <v>655000</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="17">
         <v>1</v>
       </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="19" cm="1">
+      <c r="F3" s="18"/>
+      <c r="G3" s="17" cm="1">
         <f t="array" ref="G3">C3*E3*4</f>
         <v>16</v>
       </c>
-      <c r="H3" s="21" cm="1">
+      <c r="H3" s="19" cm="1">
         <f t="array" ref="H3">G3/120</f>
-        <v>0.133333333333333</v>
-      </c>
-      <c r="I3" s="18" cm="1">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="I3" s="16" cm="1">
         <f t="array" ref="I3">C3*D3*E3</f>
         <v>2620000</v>
       </c>
-      <c r="J3" s="18" cm="1">
+      <c r="J3" s="16" cm="1">
         <f t="array" ref="J3">I3/3200</f>
         <v>818.75</v>
       </c>
-      <c r="K3" s="19">
+      <c r="K3" s="17">
         <v>4</v>
       </c>
-      <c r="L3" s="22" cm="1">
+      <c r="L3" s="20" cm="1">
         <f t="array" ref="L3">J3*K3</f>
         <v>3275</v>
       </c>
-      <c r="M3" s="22" cm="1">
+      <c r="M3" s="20" cm="1">
         <f t="array" ref="M3">L3*12</f>
         <v>39300</v>
       </c>
-      <c r="N3" s="23"/>
-      <c r="O3" s="24" cm="1">
-        <f t="array" ref="O3">'Rentabilidad'!H3</f>
-        <v>2.4625e-06</v>
-      </c>
-      <c r="P3" s="25"/>
-      <c r="Q3" t="s" s="26">
+      <c r="N3" s="21"/>
+      <c r="O3" s="22" cm="1">
+        <f t="array" ref="O3">Rentabilidad!H3</f>
+        <v>2.4625000000000001E-6</v>
+      </c>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" s="27"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="31"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="31"/>
-      <c r="Q4" s="31"/>
+    <row r="4" spans="1:17" ht="20.100000000000001" customHeight="1">
+      <c r="A4" s="25"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
     </row>
-    <row r="5" ht="44.35" customHeight="1">
-      <c r="A5" t="s" s="33">
+    <row r="5" spans="1:17" ht="44.4" customHeight="1">
+      <c r="A5" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="35">
+      <c r="B5" s="32"/>
+      <c r="C5" s="33">
         <v>4</v>
       </c>
-      <c r="D5" s="36">
+      <c r="D5" s="34">
         <v>655000</v>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="35">
         <v>2.5</v>
       </c>
-      <c r="F5" s="38"/>
-      <c r="G5" s="39" cm="1">
+      <c r="F5" s="36"/>
+      <c r="G5" s="37" cm="1">
         <f t="array" ref="G5">C5*E5*4</f>
         <v>40</v>
       </c>
-      <c r="H5" s="40" cm="1">
+      <c r="H5" s="38" cm="1">
         <f t="array" ref="H5">G5/120</f>
-        <v>0.333333333333333</v>
-      </c>
-      <c r="I5" s="36" cm="1">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="I5" s="34" cm="1">
         <f t="array" ref="I5">C5*D5*E5</f>
         <v>6550000</v>
       </c>
-      <c r="J5" s="36" cm="1">
+      <c r="J5" s="34" cm="1">
         <f t="array" ref="J5">I5/3200</f>
         <v>2046.875</v>
       </c>
-      <c r="K5" s="39">
+      <c r="K5" s="37">
         <v>4</v>
       </c>
-      <c r="L5" s="41" cm="1">
+      <c r="L5" s="39" cm="1">
         <f t="array" ref="L5">J5*K5</f>
         <v>8187.5</v>
       </c>
-      <c r="M5" s="42" cm="1">
+      <c r="M5" s="40" cm="1">
         <f t="array" ref="M5">L5*12</f>
         <v>98250</v>
       </c>
-      <c r="N5" s="43"/>
-      <c r="O5" s="44" cm="1">
-        <f t="array" ref="O5">'Rentabilidad'!H4</f>
-        <v>0.100392927308448</v>
-      </c>
-      <c r="P5" s="45"/>
-      <c r="Q5" t="s" s="26">
+      <c r="N5" s="41"/>
+      <c r="O5" s="42" cm="1">
+        <f t="array" ref="O5">Rentabilidad!H4</f>
+        <v>0.10039292730844794</v>
+      </c>
+      <c r="P5" s="43"/>
+      <c r="Q5" s="24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" ht="8.35" customHeight="1">
-      <c r="A6" s="46"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="29"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="49"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
+    <row r="6" spans="1:17" ht="8.4" customHeight="1">
+      <c r="A6" s="44"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="45"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="29"/>
+      <c r="O6" s="47"/>
+      <c r="P6" s="29"/>
+      <c r="Q6" s="29"/>
     </row>
-    <row r="7" ht="32.05" customHeight="1">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="30"/>
-      <c r="L7" t="s" s="51">
+    <row r="7" spans="1:17" ht="32.1" customHeight="1">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="52" cm="1">
+      <c r="M7" s="50" cm="1">
         <f t="array" ref="M7">M5-M3</f>
         <v>58950</v>
       </c>
-      <c r="N7" s="25"/>
-      <c r="O7" s="53"/>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="31"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="51"/>
+      <c r="P7" s="29"/>
+      <c r="Q7" s="29"/>
     </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="54"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="56"/>
-      <c r="J8" s="56"/>
-      <c r="K8" s="55"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="29"/>
-      <c r="N8" s="31"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="31"/>
+    <row r="8" spans="1:17" ht="20.100000000000001" customHeight="1">
+      <c r="A8" s="52"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="53"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="53"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="54"/>
+      <c r="K8" s="53"/>
+      <c r="L8" s="54"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="29"/>
+      <c r="O8" s="55"/>
+      <c r="P8" s="29"/>
+      <c r="Q8" s="29"/>
     </row>
-    <row r="9" ht="44.35" customHeight="1">
-      <c r="A9" t="s" s="58">
+    <row r="9" spans="1:17" ht="44.4" customHeight="1">
+      <c r="A9" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="35">
+      <c r="B9" s="32"/>
+      <c r="C9" s="33">
         <v>4</v>
       </c>
-      <c r="D9" s="59" cm="1">
-        <f t="array" ref="D9">D5+(D5*50%)</f>
-        <v>982500</v>
-      </c>
-      <c r="E9" s="37">
-        <v>2.5</v>
-      </c>
-      <c r="F9" s="38"/>
-      <c r="G9" s="39" cm="1">
+      <c r="D9" s="57">
+        <f>D5+(D5*100%)</f>
+        <v>1310000</v>
+      </c>
+      <c r="E9" s="35">
+        <v>3.5</v>
+      </c>
+      <c r="F9" s="36"/>
+      <c r="G9" s="37" cm="1">
         <f t="array" ref="G9">C9*E9*4</f>
-        <v>40</v>
-      </c>
-      <c r="H9" s="40" cm="1">
+        <v>56</v>
+      </c>
+      <c r="H9" s="38" cm="1">
         <f t="array" ref="H9">G9/120</f>
-        <v>0.333333333333333</v>
-      </c>
-      <c r="I9" s="36" cm="1">
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="I9" s="34" cm="1">
         <f t="array" ref="I9">C9*D9*E9</f>
-        <v>9825000</v>
-      </c>
-      <c r="J9" s="36" cm="1">
+        <v>18340000</v>
+      </c>
+      <c r="J9" s="34" cm="1">
         <f t="array" ref="J9">I9/3200</f>
-        <v>3070.3125</v>
-      </c>
-      <c r="K9" s="39">
+        <v>5731.25</v>
+      </c>
+      <c r="K9" s="37">
         <v>4</v>
       </c>
-      <c r="L9" s="41" cm="1">
+      <c r="L9" s="39" cm="1">
         <f t="array" ref="L9">J9*K9</f>
-        <v>12281.25</v>
-      </c>
-      <c r="M9" s="42" cm="1">
+        <v>22925</v>
+      </c>
+      <c r="M9" s="40" cm="1">
         <f t="array" ref="M9">L9*12</f>
-        <v>147375</v>
-      </c>
-      <c r="N9" s="43"/>
-      <c r="O9" s="44" cm="1">
-        <f t="array" ref="O9">'Rentabilidad'!H5</f>
-        <v>0.138607594936709</v>
-      </c>
-      <c r="P9" s="45"/>
-      <c r="Q9" t="s" s="26">
+        <v>275100</v>
+      </c>
+      <c r="N9" s="41"/>
+      <c r="O9" s="42" cm="1">
+        <f t="array" ref="O9">Rentabilidad!H5</f>
+        <v>0.32338155515370703</v>
+      </c>
+      <c r="P9" s="43"/>
+      <c r="Q9" s="24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" s="46"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="48"/>
-      <c r="K10" s="47"/>
-      <c r="L10" s="48"/>
-      <c r="M10" s="29"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="49"/>
-      <c r="P10" s="31"/>
-      <c r="Q10" s="31"/>
+    <row r="10" spans="1:17" ht="20.100000000000001" customHeight="1">
+      <c r="A10" s="44"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="29"/>
+      <c r="O10" s="47"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="29"/>
     </row>
-    <row r="11" ht="32.05" customHeight="1">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="50"/>
-      <c r="K11" s="30"/>
-      <c r="L11" t="s" s="51">
+    <row r="11" spans="1:17" ht="32.1" customHeight="1">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="60" cm="1">
+      <c r="M11" s="58" cm="1">
         <f t="array" ref="M11">M9-M3</f>
-        <v>108075</v>
-      </c>
-      <c r="N11" s="25"/>
-      <c r="O11" s="61"/>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
+        <v>235800</v>
+      </c>
+      <c r="N11" s="23"/>
+      <c r="O11" s="59"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
     </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" s="54"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="56"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="56"/>
-      <c r="J12" s="56"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="56"/>
-      <c r="M12" s="29"/>
-      <c r="N12" s="31"/>
-      <c r="O12" s="57"/>
-      <c r="P12" s="31"/>
-      <c r="Q12" s="31"/>
+    <row r="12" spans="1:17" ht="20.100000000000001" customHeight="1">
+      <c r="A12" s="52"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="53"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="53"/>
+      <c r="H12" s="53"/>
+      <c r="I12" s="54"/>
+      <c r="J12" s="54"/>
+      <c r="K12" s="53"/>
+      <c r="L12" s="54"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="29"/>
+      <c r="O12" s="55"/>
+      <c r="P12" s="29"/>
+      <c r="Q12" s="29"/>
     </row>
-    <row r="13" ht="44.35" customHeight="1">
-      <c r="A13" t="s" s="62">
+    <row r="13" spans="1:17" ht="44.4" customHeight="1">
+      <c r="A13" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="34"/>
-      <c r="C13" s="63">
-        <v>7</v>
-      </c>
-      <c r="D13" s="59" cm="1">
-        <f t="array" ref="D13">D9+(D9*50%)</f>
-        <v>1473750</v>
-      </c>
-      <c r="E13" s="37">
-        <v>2.5</v>
-      </c>
-      <c r="F13" s="38"/>
-      <c r="G13" s="39" cm="1">
+      <c r="B13" s="32"/>
+      <c r="C13" s="61">
+        <v>5</v>
+      </c>
+      <c r="D13" s="57">
+        <f>D9</f>
+        <v>1310000</v>
+      </c>
+      <c r="E13" s="35">
+        <v>3.5</v>
+      </c>
+      <c r="F13" s="36"/>
+      <c r="G13" s="37" cm="1">
         <f t="array" ref="G13">C13*E13*4</f>
         <v>70</v>
       </c>
-      <c r="H13" s="40" cm="1">
+      <c r="H13" s="38" cm="1">
         <f t="array" ref="H13">G13/120</f>
-        <v>0.583333333333333</v>
-      </c>
-      <c r="I13" s="36" cm="1">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="I13" s="34" cm="1">
         <f t="array" ref="I13">C13*D13*E13</f>
-        <v>25790625</v>
-      </c>
-      <c r="J13" s="36" cm="1">
+        <v>22925000</v>
+      </c>
+      <c r="J13" s="34" cm="1">
         <f t="array" ref="J13">I13/3200</f>
-        <v>8059.5703125</v>
-      </c>
-      <c r="K13" s="39">
+        <v>7164.0625</v>
+      </c>
+      <c r="K13" s="37">
         <v>4</v>
       </c>
-      <c r="L13" s="41" cm="1">
+      <c r="L13" s="39" cm="1">
         <f t="array" ref="L13">J13*K13</f>
-        <v>32238.28125</v>
-      </c>
-      <c r="M13" s="42" cm="1">
+        <v>28656.25</v>
+      </c>
+      <c r="M13" s="40" cm="1">
         <f t="array" ref="M13">L13*12</f>
-        <v>386859.375</v>
-      </c>
-      <c r="N13" s="43"/>
-      <c r="O13" s="44" cm="1">
-        <f t="array" ref="O13">'Rentabilidad'!H6</f>
-        <v>0.211787343215507</v>
-      </c>
-      <c r="P13" s="45"/>
-      <c r="Q13" t="s" s="26">
+        <v>343875</v>
+      </c>
+      <c r="N13" s="41"/>
+      <c r="O13" s="42" cm="1">
+        <f t="array" ref="O13">Rentabilidad!H6</f>
+        <v>0.1725769669327252</v>
+      </c>
+      <c r="P13" s="43"/>
+      <c r="Q13" s="24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" s="46"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="48"/>
-      <c r="K14" s="47"/>
-      <c r="L14" s="48"/>
-      <c r="M14" s="29"/>
-      <c r="N14" s="31"/>
-      <c r="O14" s="49"/>
-      <c r="P14" s="31"/>
-      <c r="Q14" s="31"/>
+    <row r="14" spans="1:17" ht="20.100000000000001" customHeight="1">
+      <c r="A14" s="44"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="45"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="29"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="29"/>
+      <c r="Q14" s="29"/>
     </row>
-    <row r="15" ht="44.05" customHeight="1">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="50"/>
-      <c r="K15" s="30"/>
-      <c r="L15" t="s" s="51">
+    <row r="15" spans="1:17" ht="44.1" customHeight="1">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="48"/>
+      <c r="J15" s="48"/>
+      <c r="K15" s="28"/>
+      <c r="L15" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="M15" s="64" cm="1">
+      <c r="M15" s="62" cm="1">
         <f t="array" ref="M15">M13-M7</f>
-        <v>327909.375</v>
-      </c>
-      <c r="N15" s="25"/>
-      <c r="O15" s="65"/>
-      <c r="P15" s="31"/>
-      <c r="Q15" s="31"/>
+        <v>284925</v>
+      </c>
+      <c r="N15" s="23"/>
+      <c r="O15" s="63"/>
+      <c r="P15" s="29"/>
+      <c r="Q15" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.27777800000000002" footer="0.27777800000000002"/>
+  <pageSetup scale="72" orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2546,182 +2589,182 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:H6"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="19.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="21.1172" style="66" customWidth="1"/>
-    <col min="2" max="5" width="16.3516" style="66" customWidth="1"/>
-    <col min="6" max="6" hidden="1" width="16.3333" style="66" customWidth="1"/>
-    <col min="7" max="8" width="16.3516" style="66" customWidth="1"/>
-    <col min="9" max="16384" width="16.3516" style="66" customWidth="1"/>
+    <col min="1" max="1" width="21.109375" style="5" customWidth="1"/>
+    <col min="2" max="5" width="16.33203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" style="5" hidden="1" customWidth="1"/>
+    <col min="7" max="9" width="16.33203125" style="5" customWidth="1"/>
+    <col min="10" max="16384" width="16.33203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.65" customHeight="1">
-      <c r="A1" t="s" s="7">
+    <row r="1" spans="1:8" ht="27.6" customHeight="1">
+      <c r="A1" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
     </row>
-    <row r="2" ht="30.25" customHeight="1">
-      <c r="A2" s="67"/>
-      <c r="B2" t="s" s="68">
+    <row r="2" spans="1:8" ht="30.3" customHeight="1">
+      <c r="A2" s="64"/>
+      <c r="B2" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="C2" t="s" s="68">
+      <c r="C2" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="D2" t="s" s="68">
+      <c r="D2" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="E2" t="s" s="68">
+      <c r="E2" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="F2" t="s" s="68">
+      <c r="F2" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="G2" t="s" s="68">
+      <c r="G2" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="H2" t="s" s="68">
+      <c r="H2" s="65" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" ht="21.55" customHeight="1">
-      <c r="A3" t="s" s="69">
+    <row r="3" spans="1:8" ht="21.6" customHeight="1">
+      <c r="A3" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="70">
+      <c r="B3" s="67">
         <v>2000000000</v>
       </c>
-      <c r="C3" s="71" cm="1">
+      <c r="C3" s="68" cm="1">
         <f t="array" ref="C3">B3/3200</f>
         <v>625000</v>
       </c>
-      <c r="D3" s="71" cm="1">
+      <c r="D3" s="68" cm="1">
         <f t="array" ref="D3">'Proy. X Etapas - Proyecciones f'!M3</f>
         <v>39300</v>
       </c>
-      <c r="E3" s="71" cm="1">
+      <c r="E3" s="68" cm="1">
         <f t="array" ref="E3">110000000/3200</f>
         <v>34375</v>
       </c>
-      <c r="F3" s="72" cm="1">
+      <c r="F3" s="69" cm="1">
         <f t="array" ref="F3">D3*3200</f>
         <v>125760000</v>
       </c>
-      <c r="G3" s="72" cm="1">
+      <c r="G3" s="69" cm="1">
         <f t="array" ref="G3">D3-E3</f>
         <v>4925</v>
       </c>
-      <c r="H3" s="73" cm="1">
+      <c r="H3" s="70" cm="1">
         <f t="array" ref="H3">G3/B3</f>
-        <v>2.4625e-06</v>
+        <v>2.4625000000000001E-6</v>
       </c>
     </row>
-    <row r="4" ht="21.35" customHeight="1">
-      <c r="A4" t="s" s="74">
+    <row r="4" spans="1:8" ht="21.3" customHeight="1">
+      <c r="A4" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="75">
+      <c r="B4" s="72">
         <v>36000000</v>
       </c>
-      <c r="C4" s="76" cm="1">
+      <c r="C4" s="73" cm="1">
         <f t="array" ref="C4">(B3+B4)/3200</f>
         <v>636250</v>
       </c>
-      <c r="D4" s="76" cm="1">
+      <c r="D4" s="73" cm="1">
         <f t="array" ref="D4">'Proy. X Etapas - Proyecciones f'!M5</f>
         <v>98250</v>
       </c>
-      <c r="E4" s="76" cm="1">
+      <c r="E4" s="73" cm="1">
         <f t="array" ref="E4">110000000/3200</f>
         <v>34375</v>
       </c>
-      <c r="F4" s="77" cm="1">
+      <c r="F4" s="74" cm="1">
         <f t="array" ref="F4">D4*3200</f>
         <v>314400000</v>
       </c>
-      <c r="G4" s="77" cm="1">
+      <c r="G4" s="74" cm="1">
         <f t="array" ref="G4">D4-E4</f>
         <v>63875</v>
       </c>
-      <c r="H4" s="78" cm="1">
+      <c r="H4" s="75" cm="1">
         <f t="array" ref="H4">G4/C4</f>
-        <v>0.100392927308448</v>
+        <v>0.10039292730844794</v>
       </c>
     </row>
-    <row r="5" ht="21.35" customHeight="1">
-      <c r="A5" t="s" s="74">
+    <row r="5" spans="1:8" ht="21.3" customHeight="1">
+      <c r="A5" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="75">
+      <c r="B5" s="72">
         <v>176000000</v>
       </c>
-      <c r="C5" s="76" cm="1">
+      <c r="C5" s="73" cm="1">
         <f t="array" ref="C5">(B3+B4+B5)/3200</f>
         <v>691250</v>
       </c>
-      <c r="D5" s="76" cm="1">
+      <c r="D5" s="73" cm="1">
         <f t="array" ref="D5">'Proy. X Etapas - Proyecciones f'!M9</f>
-        <v>147375</v>
-      </c>
-      <c r="E5" s="76" cm="1">
+        <v>275100</v>
+      </c>
+      <c r="E5" s="73" cm="1">
         <f t="array" ref="E5">E4*1.5</f>
         <v>51562.5</v>
       </c>
-      <c r="F5" s="77" cm="1">
+      <c r="F5" s="74" cm="1">
         <f t="array" ref="F5">D5*3200</f>
-        <v>471600000</v>
-      </c>
-      <c r="G5" s="77" cm="1">
+        <v>880320000</v>
+      </c>
+      <c r="G5" s="74" cm="1">
         <f t="array" ref="G5">D5-E5</f>
-        <v>95812.5</v>
-      </c>
-      <c r="H5" s="78" cm="1">
+        <v>223537.5</v>
+      </c>
+      <c r="H5" s="75" cm="1">
         <f t="array" ref="H5">G5/C5</f>
-        <v>0.138607594936709</v>
+        <v>0.32338155515370703</v>
       </c>
     </row>
-    <row r="6" ht="21.35" customHeight="1">
-      <c r="A6" t="s" s="74">
+    <row r="6" spans="1:8" ht="21.3" customHeight="1">
+      <c r="A6" s="71" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="75">
+      <c r="B6" s="72">
         <v>1296000000</v>
       </c>
-      <c r="C6" s="76" cm="1">
+      <c r="C6" s="73" cm="1">
         <f t="array" ref="C6">(B3+B4+B5+B6)/3200</f>
         <v>1096250</v>
       </c>
-      <c r="D6" s="76" cm="1">
+      <c r="D6" s="73" cm="1">
         <f t="array" ref="D6">'Proy. X Etapas - Proyecciones f'!M13</f>
-        <v>386859.375</v>
-      </c>
-      <c r="E6" s="76" cm="1">
+        <v>343875</v>
+      </c>
+      <c r="E6" s="73" cm="1">
         <f t="array" ref="E6">E5*3</f>
         <v>154687.5</v>
       </c>
-      <c r="F6" s="77" cm="1">
+      <c r="F6" s="74" cm="1">
         <f t="array" ref="F6">D6*3200</f>
-        <v>1237950000</v>
-      </c>
-      <c r="G6" s="77" cm="1">
+        <v>1100400000</v>
+      </c>
+      <c r="G6" s="74" cm="1">
         <f t="array" ref="G6">D6-E6</f>
-        <v>232171.875</v>
-      </c>
-      <c r="H6" s="78" cm="1">
+        <v>189187.5</v>
+      </c>
+      <c r="H6" s="75" cm="1">
         <f t="array" ref="H6">G6/C6</f>
-        <v>0.211787343215507</v>
+        <v>0.1725769669327252</v>
       </c>
     </row>
   </sheetData>
@@ -2729,7 +2772,7 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>